<commit_message>
Upfated .gutignore, Updated Project-BOM
</commit_message>
<xml_diff>
--- a/hardware/BOM_Mainboard.xlsx
+++ b/hardware/BOM_Mainboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lutzthielemann/Documents/Development/EnvNode/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE895D29-D940-3348-9EFF-F0C133E756A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{19C9FCEC-FCAC-654E-A1B3-1425776932A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37120" yWindow="2940" windowWidth="28240" windowHeight="17240" xr2:uid="{80928CA3-31BD-5C42-BF61-0691E9D1F4D9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="186" uniqueCount="125">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="193" uniqueCount="131">
   <si>
     <t>Position+A1:D13</t>
   </si>
@@ -233,9 +233,6 @@
     <t>Footprint und thermische Auslegung vor Bestückung prüfen</t>
   </si>
   <si>
-    <t>Development Board</t>
-  </si>
-  <si>
     <t>ESP32-DevKitC</t>
   </si>
   <si>
@@ -411,6 +408,27 @@
   </si>
   <si>
     <t>https://www.reichelt.de/de/de/shop/produkt/smd-widerstand_1206_100_kohm_250_mw_0_1_-238081</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>R2, R4</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>J1, J2</t>
+  </si>
+  <si>
+    <t>MCU</t>
   </si>
 </sst>
 </file>
@@ -912,19 +930,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -975,6 +988,12 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -984,12 +1003,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1009,20 +1022,20 @@
   <autoFilter ref="A1:P23" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{DE451E30-9D22-CD44-8950-489B0DB3CF00}" name="Position+A1:D13"/>
-    <tableColumn id="17" xr3:uid="{D2D340B9-BAEF-234E-8FE7-9EC0C1191319}" name="Board" dataDxfId="1"/>
+    <tableColumn id="17" xr3:uid="{D2D340B9-BAEF-234E-8FE7-9EC0C1191319}" name="Board" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{663285D9-D9B4-504D-92D8-47412D64DE7C}" name="Qty"/>
     <tableColumn id="3" xr3:uid="{3F2A56FC-27F2-DA42-BCF1-D32EDCC81854}" name="References"/>
     <tableColumn id="4" xr3:uid="{A5096E61-3BEC-E545-A3FC-4FE205EF583A}" name="Category"/>
     <tableColumn id="5" xr3:uid="{9007BB15-AB32-CF46-93C5-D4A9D08502E3}" name="Description"/>
     <tableColumn id="6" xr3:uid="{B57BE2B0-B8B1-B94A-9D66-723EADCAF285}" name="Manufacturer"/>
-    <tableColumn id="7" xr3:uid="{0AEA7C45-E829-1A4F-B5E3-BCA6E53558A6}" name="MPN" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{0AEA7C45-E829-1A4F-B5E3-BCA6E53558A6}" name="MPN" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{A502C836-37F8-0D4F-AC63-3B9A5C6AC7E6}" name="Supplier"/>
     <tableColumn id="9" xr3:uid="{BEE0F581-7C3C-CF4D-8605-81D3FAA91169}" name="Supplier_PN"/>
     <tableColumn id="10" xr3:uid="{928DD91B-22D6-0246-9450-FA705A5F3AB5}" name="URL"/>
     <tableColumn id="11" xr3:uid="{AD92798A-9943-A546-A4CE-06CB42266979}" name=" Unit_Price " dataCellStyle="Währung"/>
-    <tableColumn id="12" xr3:uid="{8D7F75CD-B994-2849-8E2B-42CD88DD23AB}" name=" Total " dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{8D7F75CD-B994-2849-8E2B-42CD88DD23AB}" name=" Total " dataDxfId="1"/>
     <tableColumn id="13" xr3:uid="{C6376C74-5C60-E543-9B24-2F6F04CCFBFB}" name="Quantity Ordered"/>
-    <tableColumn id="14" xr3:uid="{4C9D8E80-7677-C547-ABE2-192B00944580}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{4C9D8E80-7677-C547-ABE2-192B00944580}" name="Notes" dataDxfId="0"/>
     <tableColumn id="15" xr3:uid="{9AF77617-CB30-8341-80A8-3D7BFF95C930}" name="VE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1351,6 +1364,7 @@
   <cols>
     <col min="1" max="2" width="16.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="56.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" customWidth="1"/>
     <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -1365,7 +1379,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1401,387 +1415,387 @@
         <v>11</v>
       </c>
       <c r="N1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O1" t="s">
         <v>12</v>
       </c>
       <c r="P1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C2" s="4">
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2">
         <v>15</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="9"/>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="6"/>
+      <c r="I2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="L2" s="5">
+      <c r="K2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" s="4">
         <f>4.59/3</f>
         <v>1.53</v>
       </c>
-      <c r="M2" s="6">
+      <c r="M2" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>22.95</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2">
         <v>12</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="4">
+      <c r="P2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="4">
+      <c r="B3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3">
         <v>6</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="4" t="s">
+      <c r="H3" s="6"/>
+      <c r="I3" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="5">
+      <c r="L3" s="4">
         <v>0.66900000000000004</v>
       </c>
-      <c r="M3" s="6">
+      <c r="M3" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>4.0140000000000002</v>
       </c>
-      <c r="N3" s="4">
+      <c r="N3">
         <v>20</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" t="s">
         <v>21</v>
       </c>
-      <c r="P3" s="4">
+      <c r="P3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>5</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="4">
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4">
         <v>2</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="6">
         <v>10120946</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" t="s">
         <v>27</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <v>0.81</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>1.62</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4">
         <v>10</v>
       </c>
-      <c r="O4" s="4" t="s">
+      <c r="O4" t="s">
         <v>28</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>6</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="4">
+      <c r="B5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5">
         <v>2</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" t="s">
         <v>31</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" t="s">
         <v>32</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="4">
         <v>2.5499999999999998</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>5.0999999999999996</v>
       </c>
-      <c r="N5" s="4">
+      <c r="N5">
         <v>5</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>7</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="4">
+      <c r="B6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6">
         <v>4</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" t="s">
         <v>39</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" t="s">
         <v>40</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="4">
         <v>0.15</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0.6</v>
       </c>
-      <c r="N6" s="4">
+      <c r="N6">
         <v>12</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="O6" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="4">
+      <c r="B7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7">
         <v>2</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" t="s">
         <v>25</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" t="s">
         <v>46</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" t="s">
         <v>47</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="4">
         <v>0.24</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0.48</v>
       </c>
-      <c r="N7" s="4">
+      <c r="N7">
         <v>10</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="O7" t="s">
         <v>48</v>
       </c>
-      <c r="P7" s="4">
+      <c r="P7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>9</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="4">
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8">
         <v>1</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" t="s">
         <v>50</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" t="s">
         <v>52</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="4">
         <v>0.11</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0.11</v>
       </c>
-      <c r="N8" s="4">
+      <c r="N8">
         <v>10</v>
       </c>
-      <c r="O8" s="4" t="s">
+      <c r="O8" t="s">
         <v>48</v>
       </c>
-      <c r="P8" s="4">
+      <c r="P8">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A9">
         <v>10</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="4">
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9">
         <v>1</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" t="s">
         <v>53</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" t="s">
         <v>25</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" t="s">
         <v>55</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" t="s">
         <v>56</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="4">
         <v>0.28999999999999998</v>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0.28999999999999998</v>
       </c>
-      <c r="N9" s="4">
+      <c r="N9">
         <v>3</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="O9" t="s">
         <v>57</v>
       </c>
-      <c r="P9" s="4">
+      <c r="P9">
         <v>0</v>
       </c>
     </row>
@@ -1789,8 +1803,8 @@
       <c r="A10">
         <v>11</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>75</v>
+      <c r="B10" t="s">
+        <v>74</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1804,7 +1818,7 @@
       <c r="G10" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="6" t="s">
         <v>61</v>
       </c>
       <c r="I10" t="s">
@@ -1837,23 +1851,23 @@
       <c r="A11">
         <v>12</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>75</v>
+      <c r="B11" t="s">
+        <v>74</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="E11" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" t="s">
         <v>65</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>66</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>68</v>
       </c>
       <c r="L11" s="2">
         <v>5</v>
@@ -1866,7 +1880,7 @@
         <v>5</v>
       </c>
       <c r="O11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P11">
         <v>3</v>
@@ -1876,63 +1890,66 @@
       <c r="A12">
         <v>13</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>75</v>
+      <c r="B12" t="s">
+        <v>74</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
         <v>70</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>71</v>
       </c>
-      <c r="G12" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" s="8"/>
+      <c r="H12" s="6"/>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M12" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0</v>
       </c>
       <c r="O12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>14</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>76</v>
+      <c r="B13" t="s">
+        <v>75</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="D13" t="s">
+        <v>128</v>
+      </c>
+      <c r="E13" t="s">
         <v>87</v>
       </c>
-      <c r="G13" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>88</v>
+      <c r="F13" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>87</v>
       </c>
       <c r="I13" t="s">
         <v>25</v>
       </c>
       <c r="J13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L13" s="2">
         <v>0.18</v>
@@ -1950,32 +1967,32 @@
       <c r="A14">
         <v>16</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>77</v>
+      <c r="B14" t="s">
+        <v>76</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" t="s">
         <v>77</v>
       </c>
-      <c r="F14" t="s">
-        <v>78</v>
-      </c>
       <c r="G14" t="s">
-        <v>96</v>
-      </c>
-      <c r="H14" s="8">
+        <v>95</v>
+      </c>
+      <c r="H14" s="6">
         <v>333032</v>
       </c>
       <c r="I14" t="s">
         <v>25</v>
       </c>
       <c r="J14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L14" s="2">
         <v>5.3</v>
@@ -1993,32 +2010,32 @@
       <c r="A15">
         <v>17</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>83</v>
+      <c r="B15" t="s">
+        <v>82</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G15" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="8">
+        <v>95</v>
+      </c>
+      <c r="H15" s="6">
         <v>333095</v>
       </c>
       <c r="I15" t="s">
         <v>25</v>
       </c>
       <c r="J15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L15" s="2">
         <v>8.85</v>
@@ -2036,32 +2053,35 @@
       <c r="A16">
         <v>18</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>76</v>
+      <c r="B16" t="s">
+        <v>75</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
+      <c r="D16" t="s">
+        <v>127</v>
+      </c>
       <c r="E16" t="s">
         <v>35</v>
       </c>
       <c r="F16" t="s">
+        <v>120</v>
+      </c>
+      <c r="G16" t="s">
+        <v>101</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="G16" t="s">
-        <v>102</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>122</v>
       </c>
       <c r="I16" t="s">
         <v>25</v>
       </c>
       <c r="J16" t="s">
+        <v>122</v>
+      </c>
+      <c r="K16" t="s">
         <v>123</v>
-      </c>
-      <c r="K16" t="s">
-        <v>124</v>
       </c>
       <c r="L16" s="2">
         <v>0.83</v>
@@ -2079,32 +2099,35 @@
       <c r="A17">
         <v>19</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>76</v>
+      <c r="B17" t="s">
+        <v>75</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
       <c r="E17" t="s">
         <v>35</v>
       </c>
       <c r="F17" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" t="s">
         <v>103</v>
       </c>
-      <c r="G17" t="s">
-        <v>104</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>106</v>
+      <c r="H17" s="6" t="s">
+        <v>105</v>
       </c>
       <c r="I17" t="s">
         <v>25</v>
       </c>
       <c r="J17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L17" s="2">
         <v>0.06</v>
@@ -2122,32 +2145,35 @@
       <c r="A18">
         <v>20</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>76</v>
+      <c r="B18" t="s">
+        <v>75</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
+      <c r="D18" t="s">
+        <v>125</v>
+      </c>
       <c r="E18" t="s">
         <v>35</v>
       </c>
       <c r="F18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G18" t="s">
-        <v>102</v>
-      </c>
-      <c r="H18" s="8" t="s">
         <v>101</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>100</v>
       </c>
       <c r="I18" t="s">
         <v>25</v>
       </c>
       <c r="J18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L18" s="2">
         <v>0.75</v>
@@ -2162,42 +2188,44 @@
       <c r="A19">
         <v>21</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>76</v>
+      <c r="B19" t="s">
+        <v>75</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
+      <c r="D19" t="s">
+        <v>126</v>
+      </c>
       <c r="E19" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" t="s">
         <v>25</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" t="s">
         <v>47</v>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="4">
         <v>0.24</v>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0.24</v>
       </c>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4" t="s">
+      <c r="O19" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2205,32 +2233,35 @@
       <c r="A20">
         <v>22</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>76</v>
+      <c r="B20" t="s">
+        <v>75</v>
       </c>
       <c r="C20">
         <v>2</v>
       </c>
+      <c r="D20" t="s">
+        <v>129</v>
+      </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F20" t="s">
+        <v>116</v>
+      </c>
+      <c r="G20" t="s">
         <v>117</v>
       </c>
-      <c r="G20" t="s">
-        <v>118</v>
-      </c>
-      <c r="H20" s="7">
+      <c r="H20" s="5">
         <v>10120505</v>
       </c>
       <c r="I20" t="s">
         <v>25</v>
       </c>
       <c r="J20" t="s">
+        <v>118</v>
+      </c>
+      <c r="K20" t="s">
         <v>119</v>
-      </c>
-      <c r="K20" t="s">
-        <v>120</v>
       </c>
       <c r="L20" s="2">
         <v>0.31</v>
@@ -2248,32 +2279,35 @@
       <c r="A21">
         <v>23</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>76</v>
+      <c r="B21" t="s">
+        <v>75</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
+      <c r="D21" t="s">
+        <v>124</v>
+      </c>
       <c r="E21" t="s">
+        <v>107</v>
+      </c>
+      <c r="F21" t="s">
         <v>108</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>109</v>
       </c>
-      <c r="G21" t="s">
-        <v>110</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>112</v>
+      <c r="H21" s="6" t="s">
+        <v>111</v>
       </c>
       <c r="I21" t="s">
         <v>25</v>
       </c>
       <c r="J21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L21" s="2">
         <v>1.1000000000000001</v>
@@ -2288,8 +2322,8 @@
       <c r="A22">
         <v>24</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>90</v>
+      <c r="B22" t="s">
+        <v>89</v>
       </c>
       <c r="C22">
         <v>2</v>
@@ -2298,22 +2332,22 @@
         <v>22</v>
       </c>
       <c r="F22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G22" t="s">
         <v>24</v>
       </c>
-      <c r="H22" s="8" t="s">
-        <v>114</v>
+      <c r="H22" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="I22" t="s">
         <v>25</v>
       </c>
       <c r="J22" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="L22" s="2">
         <v>1.7</v>
@@ -2331,8 +2365,8 @@
       <c r="A23">
         <v>25</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>90</v>
+      <c r="B23" t="s">
+        <v>89</v>
       </c>
       <c r="C23">
         <v>12</v>
@@ -2341,9 +2375,9 @@
         <v>35</v>
       </c>
       <c r="F23" t="s">
-        <v>92</v>
-      </c>
-      <c r="H23" s="8"/>
+        <v>91</v>
+      </c>
+      <c r="H23" s="6"/>
       <c r="M23" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0</v>

</xml_diff>

<commit_message>
Fixed BOM for EnvNode and updated PCB (no breaking Changes)
</commit_message>
<xml_diff>
--- a/hardware/BOM_Mainboard.xlsx
+++ b/hardware/BOM_Mainboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lutzthielemann/Documents/Development/EnvNode/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{19C9FCEC-FCAC-654E-A1B3-1425776932A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{50CC93AA-54CC-0141-AFC7-04BEB41E1CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37120" yWindow="2940" windowWidth="28240" windowHeight="17240" xr2:uid="{80928CA3-31BD-5C42-BF61-0691E9D1F4D9}"/>
+    <workbookView xWindow="-29520" yWindow="1980" windowWidth="28240" windowHeight="17240" xr2:uid="{80928CA3-31BD-5C42-BF61-0691E9D1F4D9}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_Mainboard" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="193" uniqueCount="131">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="211" uniqueCount="143">
   <si>
     <t>Position+A1:D13</t>
   </si>
@@ -125,9 +125,6 @@
     <t>Für interne Qwiic-Breakouts; Bauhöhe und Ausführung passend zur Mechanik wählen</t>
   </si>
   <si>
-    <t>PinSocket 1x19, 2.54mm</t>
-  </si>
-  <si>
     <t>BL1.20 G</t>
   </si>
   <si>
@@ -429,6 +426,45 @@
   </si>
   <si>
     <t>MCU</t>
+  </si>
+  <si>
+    <t>GPIO's</t>
+  </si>
+  <si>
+    <t>I2CA0 1-3  I2C1 1-3</t>
+  </si>
+  <si>
+    <t>I2C0 4, I2C1 4</t>
+  </si>
+  <si>
+    <t>ESP32</t>
+  </si>
+  <si>
+    <t>PinSocket 1x20, 2.54mm, cut to 19 Pins</t>
+  </si>
+  <si>
+    <t>C3, C4</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>JST - Stiftleiste, gerade, 1x2-polig - PH</t>
+  </si>
+  <si>
+    <t>B2B-PH-K-S</t>
+  </si>
+  <si>
+    <t>JST PH2P ST</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.de/de/de/shop/produkt/jst_-_stiftleiste_gerade_1x2-polig_-_ph-185049</t>
   </si>
 </sst>
 </file>
@@ -1018,8 +1054,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}" name="Tabelle1" displayName="Tabelle1" ref="A1:P23" totalsRowShown="0">
-  <autoFilter ref="A1:P23" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}"/>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}" name="Tabelle1" displayName="Tabelle1" ref="A1:P24" totalsRowShown="0">
+  <autoFilter ref="A1:P24" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{DE451E30-9D22-CD44-8950-489B0DB3CF00}" name="Position+A1:D13"/>
     <tableColumn id="17" xr3:uid="{D2D340B9-BAEF-234E-8FE7-9EC0C1191319}" name="Board" dataDxfId="3"/>
@@ -1359,7 +1395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32D7DD83-8DEB-2D43-B6AF-9C9D802E4658}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="16.83203125" customWidth="1"/>
@@ -1379,7 +1415,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1415,13 +1451,13 @@
         <v>11</v>
       </c>
       <c r="N1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O1" t="s">
         <v>12</v>
       </c>
       <c r="P1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -1429,10 +1465,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C2">
         <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>130</v>
       </c>
       <c r="E2" t="s">
         <v>13</v>
@@ -1448,7 +1487,7 @@
         <v>19</v>
       </c>
       <c r="K2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L2" s="4">
         <f>4.59/3</f>
@@ -1473,10 +1512,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>131</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -1516,10 +1558,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4">
         <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>132</v>
       </c>
       <c r="E4" t="s">
         <v>22</v>
@@ -1564,31 +1609,34 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
+      <c r="D5" t="s">
+        <v>133</v>
+      </c>
       <c r="E5" t="s">
         <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>134</v>
       </c>
       <c r="G5" t="s">
         <v>24</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I5" t="s">
         <v>25</v>
       </c>
       <c r="J5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" t="s">
         <v>31</v>
-      </c>
-      <c r="K5" t="s">
-        <v>32</v>
       </c>
       <c r="L5" s="4">
         <v>2.5499999999999998</v>
@@ -1601,7 +1649,7 @@
         <v>5</v>
       </c>
       <c r="O5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -1609,34 +1657,34 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
         <v>34</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="I6" t="s">
         <v>25</v>
       </c>
       <c r="J6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" t="s">
         <v>39</v>
-      </c>
-      <c r="K6" t="s">
-        <v>40</v>
       </c>
       <c r="L6" s="4">
         <v>0.15</v>
@@ -1649,7 +1697,7 @@
         <v>12</v>
       </c>
       <c r="O6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1660,31 +1708,34 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
+      <c r="D7" t="s">
+        <v>135</v>
+      </c>
       <c r="E7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
         <v>42</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>45</v>
       </c>
       <c r="I7" t="s">
         <v>25</v>
       </c>
       <c r="J7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K7" t="s">
         <v>46</v>
-      </c>
-      <c r="K7" t="s">
-        <v>47</v>
       </c>
       <c r="L7" s="4">
         <v>0.24</v>
@@ -1697,7 +1748,7 @@
         <v>10</v>
       </c>
       <c r="O7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P7">
         <v>10</v>
@@ -1708,31 +1759,34 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
+      <c r="D8" t="s">
+        <v>125</v>
+      </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" t="s">
         <v>49</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>51</v>
       </c>
       <c r="I8" t="s">
         <v>25</v>
       </c>
       <c r="J8" t="s">
+        <v>50</v>
+      </c>
+      <c r="K8" t="s">
         <v>51</v>
-      </c>
-      <c r="K8" t="s">
-        <v>52</v>
       </c>
       <c r="L8" s="4">
         <v>0.11</v>
@@ -1745,7 +1799,7 @@
         <v>10</v>
       </c>
       <c r="O8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P8">
         <v>10</v>
@@ -1756,31 +1810,34 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
+      <c r="D9" t="s">
+        <v>136</v>
+      </c>
       <c r="E9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="G9" t="s">
-        <v>50</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I9" t="s">
         <v>25</v>
       </c>
       <c r="J9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K9" t="s">
         <v>55</v>
-      </c>
-      <c r="K9" t="s">
-        <v>56</v>
       </c>
       <c r="L9" s="4">
         <v>0.28999999999999998</v>
@@ -1793,7 +1850,7 @@
         <v>3</v>
       </c>
       <c r="O9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1804,31 +1861,34 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
+      <c r="D10" t="s">
+        <v>123</v>
+      </c>
       <c r="E10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
         <v>58</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>59</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="I10" t="s">
         <v>25</v>
       </c>
       <c r="J10" t="s">
+        <v>61</v>
+      </c>
+      <c r="K10" t="s">
         <v>62</v>
-      </c>
-      <c r="K10" t="s">
-        <v>63</v>
       </c>
       <c r="L10" s="2">
         <v>1</v>
@@ -1841,7 +1901,7 @@
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P10">
         <v>3</v>
@@ -1852,22 +1912,25 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
+      <c r="D11" t="s">
+        <v>137</v>
+      </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
         <v>65</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" s="6" t="s">
         <v>66</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>67</v>
       </c>
       <c r="L11" s="2">
         <v>5</v>
@@ -1880,7 +1943,7 @@
         <v>5</v>
       </c>
       <c r="O11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P11">
         <v>3</v>
@@ -1891,30 +1954,30 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="E12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" t="s">
         <v>69</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>70</v>
-      </c>
-      <c r="G12" t="s">
-        <v>71</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M12" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0</v>
       </c>
       <c r="O12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -1922,127 +1985,126 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E13" t="s">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>86</v>
+        <v>139</v>
       </c>
       <c r="G13" t="s">
-        <v>93</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>87</v>
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>140</v>
       </c>
       <c r="I13" t="s">
         <v>25</v>
       </c>
       <c r="J13" t="s">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="K13" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
       <c r="L13" s="2">
-        <v>0.18</v>
+        <v>1.3</v>
       </c>
       <c r="M13" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>0.18</v>
-      </c>
-      <c r="N13">
-        <v>5</v>
-      </c>
-      <c r="O13" s="1"/>
+        <v>1.3</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
+      <c r="D14" t="s">
+        <v>127</v>
+      </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H14" s="6">
-        <v>333032</v>
+        <v>92</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="I14" t="s">
         <v>25</v>
       </c>
       <c r="J14" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="K14" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L14" s="2">
-        <v>5.3</v>
+        <v>0.18</v>
       </c>
       <c r="M14" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>5.3</v>
+        <v>0.18</v>
       </c>
       <c r="N14">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O14" s="1"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H15" s="6">
-        <v>333095</v>
+        <v>333032</v>
       </c>
       <c r="I15" t="s">
         <v>25</v>
       </c>
       <c r="J15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="K15" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L15" s="2">
-        <v>8.85</v>
+        <v>5.3</v>
       </c>
       <c r="M15" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>8.85</v>
+        <v>5.3</v>
       </c>
       <c r="N15">
         <v>1</v>
@@ -2051,346 +2113,389 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C16">
-        <v>2</v>
-      </c>
-      <c r="D16" t="s">
-        <v>127</v>
+        <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>35</v>
+        <v>82</v>
       </c>
       <c r="F16" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
       <c r="G16" t="s">
-        <v>101</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>121</v>
+        <v>94</v>
+      </c>
+      <c r="H16" s="6">
+        <v>333095</v>
       </c>
       <c r="I16" t="s">
         <v>25</v>
       </c>
       <c r="J16" t="s">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="K16" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="L16" s="2">
-        <v>0.83</v>
+        <v>8.85</v>
       </c>
       <c r="M16" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>1.66</v>
+        <v>8.85</v>
       </c>
       <c r="N16">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="s">
+        <v>126</v>
+      </c>
+      <c r="E17" t="s">
         <v>34</v>
       </c>
-      <c r="E17" t="s">
-        <v>35</v>
-      </c>
       <c r="F17" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="G17" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="I17" t="s">
         <v>25</v>
       </c>
       <c r="J17" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="K17" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="L17" s="2">
-        <v>0.06</v>
+        <v>0.83</v>
       </c>
       <c r="M17" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>0.06</v>
+        <v>1.66</v>
       </c>
       <c r="N17">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="O17" s="1"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>125</v>
+        <v>33</v>
       </c>
       <c r="E18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F18" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I18" t="s">
         <v>25</v>
       </c>
       <c r="J18" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K18" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="L18" s="2">
-        <v>0.75</v>
+        <v>0.06</v>
       </c>
       <c r="M18" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>0.75</v>
+        <v>0.06</v>
+      </c>
+      <c r="N18">
+        <v>50</v>
       </c>
       <c r="O18" s="1"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E19" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="G19" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="I19" t="s">
         <v>25</v>
       </c>
       <c r="J19" t="s">
-        <v>46</v>
+        <v>98</v>
       </c>
       <c r="K19" t="s">
-        <v>47</v>
-      </c>
-      <c r="L19" s="4">
-        <v>0.24</v>
+        <v>97</v>
+      </c>
+      <c r="L19" s="2">
+        <v>0.75</v>
       </c>
       <c r="M19" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>0.24</v>
-      </c>
-      <c r="O19" t="s">
-        <v>48</v>
-      </c>
+        <v>0.75</v>
+      </c>
+      <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="1:15" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E20" t="s">
-        <v>90</v>
+        <v>41</v>
       </c>
       <c r="F20" t="s">
-        <v>116</v>
+        <v>42</v>
       </c>
       <c r="G20" t="s">
-        <v>117</v>
-      </c>
-      <c r="H20" s="5">
-        <v>10120505</v>
+        <v>43</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>44</v>
       </c>
       <c r="I20" t="s">
         <v>25</v>
       </c>
       <c r="J20" t="s">
-        <v>118</v>
+        <v>45</v>
       </c>
       <c r="K20" t="s">
-        <v>119</v>
-      </c>
-      <c r="L20" s="2">
-        <v>0.31</v>
+        <v>46</v>
+      </c>
+      <c r="L20" s="4">
+        <v>0.24</v>
       </c>
       <c r="M20" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>0.62</v>
-      </c>
-      <c r="N20">
-        <v>20</v>
-      </c>
-      <c r="O20" s="1"/>
+        <v>0.24</v>
+      </c>
+      <c r="O20" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="F21" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="G21" t="s">
-        <v>109</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>111</v>
+        <v>116</v>
+      </c>
+      <c r="H21" s="5">
+        <v>10120505</v>
       </c>
       <c r="I21" t="s">
         <v>25</v>
       </c>
       <c r="J21" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="K21" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="L21" s="2">
-        <v>1.1000000000000001</v>
+        <v>0.31</v>
       </c>
       <c r="M21" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>1.1000000000000001</v>
+        <v>0.62</v>
+      </c>
+      <c r="N21">
+        <v>20</v>
       </c>
       <c r="O21" s="1"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>123</v>
       </c>
       <c r="E22" t="s">
-        <v>22</v>
+        <v>106</v>
       </c>
       <c r="F22" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="G22" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I22" t="s">
         <v>25</v>
       </c>
       <c r="J22" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="K22" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L22" s="2">
-        <v>1.7</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="M22" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
-        <v>3.4</v>
-      </c>
-      <c r="N22">
-        <v>2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23">
+        <v>24</v>
+      </c>
+      <c r="B23" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I23" t="s">
         <v>25</v>
       </c>
-      <c r="B23" t="s">
-        <v>89</v>
-      </c>
-      <c r="C23">
-        <v>12</v>
-      </c>
-      <c r="E23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" t="s">
-        <v>91</v>
-      </c>
-      <c r="H23" s="6"/>
+      <c r="J23" t="s">
+        <v>114</v>
+      </c>
+      <c r="K23" t="s">
+        <v>113</v>
+      </c>
+      <c r="L23" s="2">
+        <v>1.7</v>
+      </c>
       <c r="M23" s="3">
         <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
+        <v>3.4</v>
+      </c>
+      <c r="N23">
+        <v>2</v>
+      </c>
+      <c r="O23" s="1"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" t="s">
+        <v>90</v>
+      </c>
+      <c r="H24" s="6"/>
+      <c r="M24" s="3">
+        <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
         <v>0</v>
       </c>
-      <c r="N23">
+      <c r="N24">
         <v>12</v>
       </c>
-      <c r="O23" s="1"/>
+      <c r="O24" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="K22" r:id="rId1" location="open-modal-image-big-slider" xr:uid="{55EF9935-EEF8-7246-8701-F9DFC3DEFC41}"/>
+    <hyperlink ref="K23" r:id="rId1" location="open-modal-image-big-slider" xr:uid="{55EF9935-EEF8-7246-8701-F9DFC3DEFC41}"/>
   </hyperlinks>
   <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Updated BOM for Relay
</commit_message>
<xml_diff>
--- a/hardware/BOM_Mainboard.xlsx
+++ b/hardware/BOM_Mainboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lutzthielemann/Documents/Development/EnvNode/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{50CC93AA-54CC-0141-AFC7-04BEB41E1CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2A232CCE-33AB-CD40-A521-A3BE9E35D7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-29520" yWindow="1980" windowWidth="28240" windowHeight="17240" xr2:uid="{80928CA3-31BD-5C42-BF61-0691E9D1F4D9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="211" uniqueCount="143">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="220" uniqueCount="150">
   <si>
     <t>Position+A1:D13</t>
   </si>
@@ -465,6 +465,27 @@
   </si>
   <si>
     <t>https://www.reichelt.de/de/de/shop/produkt/jst_-_stiftleiste_gerade_1x2-polig_-_ph-185049</t>
+  </si>
+  <si>
+    <t>Relay</t>
+  </si>
+  <si>
+    <t>K1, K2</t>
+  </si>
+  <si>
+    <t>Steck-Printrelais, 1 CO, 6 A, 5 V DC sensitiv</t>
+  </si>
+  <si>
+    <t>finder</t>
+  </si>
+  <si>
+    <t>34.51.7.005.0010</t>
+  </si>
+  <si>
+    <t>FIN 34.51.7 5V</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.de/de/de/shop/produkt/steck-printrelais_1_co_6_a_5_v_dc_sensitiv-259179?PROVID=2788&amp;gad_source=1&amp;gad_campaignid=21154720511&amp;gbraid=0AAAAADwnxtb50MtqKwtKae8MAeGQARqWX&amp;gclid=CjwKCAjw7p_UBhBlEiwAhpIs72D6cK8XQyuxcrvb0uftoYY3618BT3lTyYSWWSou1J99G9udBcpsbhoCJbcQAvD_BwE</t>
   </si>
 </sst>
 </file>
@@ -966,7 +987,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -976,6 +997,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20 % - Akzent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -1054,8 +1076,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}" name="Tabelle1" displayName="Tabelle1" ref="A1:P24" totalsRowShown="0">
-  <autoFilter ref="A1:P24" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}"/>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}" name="Tabelle1" displayName="Tabelle1" ref="A1:P25" totalsRowShown="0">
+  <autoFilter ref="A1:P25" xr:uid="{08C33A7F-931E-3844-8522-09F575F12B8C}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{DE451E30-9D22-CD44-8950-489B0DB3CF00}" name="Position+A1:D13"/>
     <tableColumn id="17" xr3:uid="{D2D340B9-BAEF-234E-8FE7-9EC0C1191319}" name="Board" dataDxfId="3"/>
@@ -1395,7 +1417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32D7DD83-8DEB-2D43-B6AF-9C9D802E4658}">
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="16.83203125" customWidth="1"/>
@@ -2382,7 +2404,7 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>74</v>
@@ -2425,7 +2447,7 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>88</v>
@@ -2468,7 +2490,7 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>88</v>
@@ -2491,6 +2513,49 @@
         <v>12</v>
       </c>
       <c r="O24" s="1"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" t="s">
+        <v>143</v>
+      </c>
+      <c r="F25" t="s">
+        <v>145</v>
+      </c>
+      <c r="G25" t="s">
+        <v>146</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="I25" t="s">
+        <v>25</v>
+      </c>
+      <c r="J25" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" t="s">
+        <v>149</v>
+      </c>
+      <c r="L25" s="2">
+        <v>5.8</v>
+      </c>
+      <c r="M25" s="3">
+        <f>Tabelle1[[#This Row],[Qty]]*Tabelle1[[#This Row],[ Unit_Price ]]</f>
+        <v>11.6</v>
+      </c>
+      <c r="O25" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>

</xml_diff>